<commit_message>
feat: enhance ScanWindow with auto-attendance functionality and visual feedback for successful scans
</commit_message>
<xml_diff>
--- a/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
+++ b/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
@@ -642,9 +642,21 @@
           <t>null 4</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>12:41:30 AM</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>yti</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -765,8 +777,16 @@
           <t>null 7</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>12:41:32 AM</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
@@ -810,9 +830,21 @@
           <t>null 8</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>12:41:33 AM</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>[01:16:09 AM] Canceled.</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -855,9 +887,21 @@
           <t>null 9</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>12:41:34 AM</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>[01:16:06 AM] Canceled.</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -900,8 +944,16 @@
           <t>null 10</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>12:41:36 AM</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
@@ -945,8 +997,16 @@
           <t>null 11</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>12:41:37 AM</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
@@ -991,8 +1051,16 @@
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>12:41:38 AM</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>[01:14:52 AM] Canceled.</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1035,8 +1103,16 @@
           <t>null 13</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>12:41:39 AM</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
@@ -1080,8 +1156,16 @@
           <t>null 14</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>12:41:40 AM</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
@@ -1125,8 +1209,16 @@
           <t>null 15</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>12:41:42 AM</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
@@ -1252,8 +1344,16 @@
           <t>null 18</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>12:42:19 AM</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
@@ -1297,8 +1397,16 @@
           <t>null 19</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>12:42:17 AM</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
@@ -1342,8 +1450,16 @@
           <t>null 20</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>01:06:37 AM</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
@@ -1387,8 +1503,16 @@
           <t>null 21</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>01:06:43 AM</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
@@ -1432,8 +1556,16 @@
           <t>null 22</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>01:06:48 AM</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
@@ -1477,8 +1609,16 @@
           <t>null 23</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>01:06:50 AM</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
@@ -1522,8 +1662,16 @@
           <t>null 24</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>01:06:53 AM</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
@@ -1567,8 +1715,16 @@
           <t>null 25</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>01:06:57 AM</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
@@ -1687,8 +1843,16 @@
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>01:07:32 AM</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>[01:07:32 AM] Canceled.</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1731,8 +1895,16 @@
           <t>null 29</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>01:07:21 AM</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
@@ -1859,8 +2031,17 @@
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>01:08:05 AM</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>[01:08:05 AM] Canceled.
+[01:14:39 AM] Canceled.</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1903,8 +2084,16 @@
           <t>null 33</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>01:08:01 AM</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
@@ -1948,8 +2137,16 @@
           <t>null 34</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>01:08:03 AM</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
@@ -2068,8 +2265,16 @@
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>01:14:22 AM</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>[01:14:47 AM] Canceled.</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -2112,8 +2317,16 @@
           <t>null 38</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>01:14:23 AM</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
@@ -2157,8 +2370,16 @@
           <t>null 39</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>01:14:44 AM</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
@@ -2202,8 +2423,16 @@
           <t>null 40</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>01:15:30 AM</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
@@ -2247,8 +2476,16 @@
           <t>null 41</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>01:15:39 AM</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
@@ -2292,8 +2529,16 @@
           <t>null 42</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>01:15:40 AM</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add grade normalization and validation functions in ScanWindow
</commit_message>
<xml_diff>
--- a/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
+++ b/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
@@ -887,11 +887,7 @@
           <t>null 9</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>12:41:34 AM</t>
@@ -899,7 +895,8 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>[01:16:06 AM] Canceled.</t>
+          <t>[01:16:06 AM] Canceled.
+[01:39:30 AM] Canceled.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2582,8 +2579,16 @@
           <t>null 43</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>01:28:05 AM</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
@@ -2627,8 +2632,16 @@
           <t>null 44</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>01:28:06 AM</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
@@ -2672,8 +2685,16 @@
           <t>null 45</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>01:28:08 AM</t>
+        </is>
+      </c>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
@@ -2717,8 +2738,16 @@
           <t>null 46</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>01:28:13 AM</t>
+        </is>
+      </c>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
@@ -2762,8 +2791,16 @@
           <t>null 47</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>01:28:25 AM</t>
+        </is>
+      </c>
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
@@ -2807,9 +2844,21 @@
           <t>null 48</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>01:28:26 AM</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>khlkj</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr">
         <is>
           <t>excel_import</t>

</xml_diff>

<commit_message>
refactor session management and update UI components
</commit_message>
<xml_diff>
--- a/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
+++ b/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
@@ -699,9 +699,21 @@
           <t>null 5</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>05:28:01 AM</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>[05:28:01 AM] Attended (Didn't do Exam &amp; Homework).</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1047,7 +1059,11 @@
           <t>null 12</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>12:41:38 AM</t>
@@ -1055,7 +1071,8 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>[01:14:52 AM] Canceled.</t>
+          <t>[01:14:52 AM] Canceled.
+[05:27:42 AM] Canceled.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1259,9 +1276,21 @@
           <t>null 16</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>05:27:54 AM</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>[05:27:54 AM] Completed Exam &amp; Homework at center.</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1296,8 +1325,16 @@
           <t>null 17</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>05:28:27 AM</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
@@ -1945,8 +1982,16 @@
           <t>null 30</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>05:28:52 AM</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
@@ -2261,7 +2306,11 @@
           <t>null 37</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr">
         <is>
           <t>01:14:22 AM</t>
@@ -2901,8 +2950,16 @@
           <t>null 49</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>05:27:15 AM</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
@@ -3028,8 +3085,16 @@
           <t>null 52</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>05:28:57 AM</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
@@ -3151,8 +3216,16 @@
           <t>null 55</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>05:28:59 AM</t>
+        </is>
+      </c>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
@@ -3196,8 +3269,16 @@
           <t>null 56</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>05:29:04 AM</t>
+        </is>
+      </c>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
@@ -3241,8 +3322,16 @@
           <t>null 57</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>05:29:11 AM</t>
+        </is>
+      </c>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add unit tests for session logic and related functionalities
- Implement tests for focus view state formatting, filter application, and grade logic handling.
- Validate attendance update preservation and manual record addition.
- Ensure proper handling of missing tasks and scan context marking.
- Test row matching against filters and focus action payload construction.
- Verify session summary computation and record addition behavior.
- Include duplicate lookup tests for session manager using mapping.
</commit_message>
<xml_diff>
--- a/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
+++ b/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
@@ -425,63 +425,73 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Student ID</t>
+          <t>student id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>phone</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Parent Phone</t>
+          <t>parent phone</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Card ID</t>
+          <t>card id</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Attendance Status</t>
+          <t>attendance status</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Timestamp (e.g. 2024-07-05 14:30:00)</t>
+          <t>timestamp (e.g. 2024-07-05 14:30:00)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>note</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Attendance Method</t>
+          <t>attendance method</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Exam 1 (Homework)</t>
+          <t>exam 1 (homework)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Exam 2 (Quiz)</t>
+          <t>exam 2 (quiz)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>_manual_added</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>_last_action</t>
         </is>
       </c>
     </row>
@@ -493,7 +503,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>سلمى ابراهيم</t>
+          <t>ﻢﻴﻫﺍﺮﺑﺍ ﻰﻤﻠﺳ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -511,9 +521,21 @@
           <t>null 1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>06:05:44 AM</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>[06:05:44 AM] Attended (Didn't do Exam &amp; Homework).rtzufxufu</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -521,6 +543,12 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -548,8 +576,16 @@
           <t>null 2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>06:05:55 AM</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
@@ -566,6 +602,12 @@
           <t>9/10</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -615,6 +657,8 @@
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -672,6 +716,8 @@
           <t>10/10</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -721,6 +767,8 @@
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -762,6 +810,8 @@
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -815,6 +865,8 @@
           <t>9/10</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -872,6 +924,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -926,6 +980,8 @@
           <t>9/10</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -979,6 +1035,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1032,6 +1090,8 @@
           <t>5/10</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1090,6 +1150,8 @@
           <t>6/10</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1143,6 +1205,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1196,6 +1260,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1249,6 +1315,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1298,6 +1366,8 @@
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1351,6 +1421,8 @@
           <t>2/10</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1404,6 +1476,8 @@
           <t>5/10</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1457,6 +1531,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1510,6 +1586,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1563,6 +1641,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1616,6 +1696,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1669,6 +1751,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1722,6 +1806,8 @@
           <t>5/10</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1775,6 +1861,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1812,6 +1900,8 @@
       </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1849,6 +1939,8 @@
       </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1902,6 +1994,8 @@
           <t>3/10</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1955,6 +2049,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2008,6 +2104,8 @@
           <t>9/10</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2045,6 +2143,8 @@
       </c>
       <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2099,6 +2199,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2152,6 +2254,8 @@
           <t>6/10</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2205,6 +2309,8 @@
           <t>6/10</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2242,6 +2348,8 @@
       </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2279,6 +2387,8 @@
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2336,6 +2446,8 @@
           <t>5/10</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2389,6 +2501,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2442,6 +2556,8 @@
           <t>5/10</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2495,6 +2611,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2548,6 +2666,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2601,6 +2721,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2654,6 +2776,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2707,6 +2831,8 @@
           <t>1/10</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2760,6 +2886,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2813,6 +2941,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2866,6 +2996,8 @@
           <t>10/10</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2923,6 +3055,8 @@
           <t>9/10</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2976,6 +3110,8 @@
           <t>9/10</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3021,6 +3157,8 @@
           <t>5/10</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3058,6 +3196,8 @@
       </c>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3111,6 +3251,8 @@
           <t>9/10</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3152,6 +3294,8 @@
         </is>
       </c>
       <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3189,6 +3333,8 @@
       </c>
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3242,6 +3388,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3295,6 +3443,8 @@
           <t>6/10</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3348,6 +3498,8 @@
           <t>5/10</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3393,6 +3545,8 @@
           <t>4/10</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3438,6 +3592,8 @@
           <t>2/10</t>
         </is>
       </c>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3483,6 +3639,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3528,6 +3686,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3569,6 +3729,8 @@
         </is>
       </c>
       <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3606,6 +3768,8 @@
       </c>
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3643,6 +3807,8 @@
       </c>
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3688,6 +3854,8 @@
           <t>6/10</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3733,6 +3901,8 @@
           <t>6/10</t>
         </is>
       </c>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3778,6 +3948,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3823,6 +3995,8 @@
           <t>9/10</t>
         </is>
       </c>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3868,6 +4042,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3913,6 +4089,8 @@
           <t>7/10</t>
         </is>
       </c>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3950,6 +4128,8 @@
       </c>
       <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3995,6 +4175,8 @@
           <t>6/10</t>
         </is>
       </c>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4040,6 +4222,8 @@
           <t>9/10</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4085,6 +4269,8 @@
           <t>9/10</t>
         </is>
       </c>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4130,6 +4316,8 @@
           <t>6/10</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4171,6 +4359,8 @@
         </is>
       </c>
       <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4216,6 +4406,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4253,6 +4445,8 @@
       </c>
       <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4298,6 +4492,8 @@
           <t>5/10</t>
         </is>
       </c>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4343,6 +4539,8 @@
           <t>9/10</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4388,6 +4586,8 @@
           <t>5/10</t>
         </is>
       </c>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4433,6 +4633,8 @@
           <t>6/10</t>
         </is>
       </c>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4478,6 +4680,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4523,6 +4727,8 @@
           <t>5/10</t>
         </is>
       </c>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4560,6 +4766,8 @@
       </c>
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4597,6 +4805,8 @@
       </c>
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4642,6 +4852,8 @@
           <t>8/10</t>
         </is>
       </c>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4683,6 +4895,8 @@
           <t>6/10</t>
         </is>
       </c>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4724,6 +4938,8 @@
         </is>
       </c>
       <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4761,6 +4977,8 @@
       </c>
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4798,6 +5016,8 @@
       </c>
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4843,6 +5063,8 @@
           <t>6/10</t>
         </is>
       </c>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4888,6 +5110,8 @@
           <t>5/10</t>
         </is>
       </c>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4925,6 +5149,8 @@
       </c>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4958,6 +5184,8 @@
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4995,6 +5223,8 @@
         </is>
       </c>
       <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Enhance focus view note handling and persistence in ScanWindow
</commit_message>
<xml_diff>
--- a/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
+++ b/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
@@ -1892,7 +1892,11 @@
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>5ueu</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1931,7 +1935,11 @@
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>aetujsertset</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>excel_import</t>

</xml_diff>

<commit_message>
Add queue status handling and global scan shortcuts in ScanWindow
</commit_message>
<xml_diff>
--- a/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
+++ b/Sessions/test/3rd/Ferdous/3rd Ferdous session 1.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>[06:05:44 AM] Attended (Didn't do Exam &amp; Homework).rtzufxufu</t>
+          <t>[06:05:44 AM] Attended (Didn't do Exam &amp; Homework).rtzufxufun</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -576,17 +576,17 @@
           <t>null 2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>06:05:55 AM</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>06:51:40 AM</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>[06:51:40 AM] Canceled.</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -605,7 +605,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>attend</t>
+          <t>canceled</t>
         </is>
       </c>
     </row>
@@ -635,19 +635,16 @@
           <t>null 3</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>12:31:47 AM</t>
+          <t>06:46:16 AM</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>[12:31:47 AM] Attended (Didn't do Exam &amp; Homework).</t>
+          <t>[12:31:47 AM] Attended (Didn't do Exam &amp; Homework).
+[06:46:16 AM] Canceled.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -658,7 +655,11 @@
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>canceled</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -668,7 +669,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>مروان هاني</t>
+          <t>ﻲﻧﺎﻫ ﻥﺍﻭﺮﻣ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -686,19 +687,16 @@
           <t>null 4</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>12:41:30 AM</t>
+          <t>06:46:18 AM</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>yti</t>
+          <t>yti
+[06:46:18 AM] Canceled.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -717,7 +715,11 @@
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>canceled</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1046,7 +1048,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>على شاكر سمير</t>
+          <t>ﺮﻴﻤﺳ ﺮﻛﺎﺷ ﻰﻠﻋ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1064,17 +1066,17 @@
           <t>null 11</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>attend</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>12:41:37 AM</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>06:51:42 AM</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>[06:51:42 AM] Canceled.</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>excel_import</t>
@@ -1091,7 +1093,11 @@
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>canceled</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3147,8 +3153,16 @@
           <t>null 50</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>06:47:42 AM</t>
+        </is>
+      </c>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
@@ -3166,7 +3180,11 @@
         </is>
       </c>
       <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>attend</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">

</xml_diff>